<commit_message>
Add PHP review app on a normalized content DB
- Content DB: normalized schema (scripts/schema.sql) with stable keys for
  masail, readings, mawadi; plain-text search columns; qiraat_v view
- Row-level agreement with Hafs (same lafz and ada' in an overlapping hal)
- app/: browse/filter by qari or rawi, sura/aya range, bab, hal, khilaf;
  wide table, masala pages, matn browser, CSV export
- Review workflow: reviewers flag any masala/reading/mawdi/rawi-reading/bayt,
  admins accept/reject with discussion, export accepted as JSON;
  scripts/reviews.py turns the export into a YAML checklist
- Apply confirmed rulings: idgham kabir for Susi; imala of al-nas for Douri;
  both wujuh for Qalun in al-da'i/da'ani with hadhf more famous

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/out/riwayat/ابن كثير.xlsx
+++ b/data/out/riwayat/ابن كثير.xlsx
@@ -597,7 +597,7 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -729,7 +729,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -3765,7 +3765,7 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3897,7 +3897,7 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4293,7 +4293,7 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4425,7 +4425,7 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -5085,7 +5085,7 @@
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -5217,7 +5217,7 @@
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -5349,7 +5349,7 @@
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -5481,7 +5481,7 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -10827,7 +10827,7 @@
       <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -10893,7 +10893,7 @@
       <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -11421,7 +11421,7 @@
       <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -11553,7 +11553,7 @@
       <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
-          <t>لا</t>
+          <t>نعم</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">

</xml_diff>

<commit_message>
2-m05: imala of al-nas (majrur) for Douri alone; drop the fath wajh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/out/riwayat/ابن كثير.xlsx
+++ b/data/out/riwayat/ابن كثير.xlsx
@@ -2130,7 +2130,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>مفهوم: الخلاف لمن ذُكر</t>
+          <t>مفهوم: الإمالة لمن ذُكر</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>مفهوم: الخلاف لمن ذُكر</t>
+          <t>مفهوم: الإمالة لمن ذُكر</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">

</xml_diff>